<commit_message>
AI Audit log week 2
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenVietKhanh_DE181002.xlsx
+++ b/AI Audit Log_NguyenVietKhanh_DE181002.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MYPC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\AI_Log\ai-audit-log-KhanhNV1374\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C495412D-220C-4D07-B45D-30E1DB914200}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F792AFA-9814-438F-B786-258B6D5AC9A3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="1" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="2" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -147,6 +147,96 @@
   </si>
   <si>
     <t>Architecture Analysis</t>
+  </si>
+  <si>
+    <t>Requirement Analysis</t>
+  </si>
+  <si>
+    <t>What actors and use cases are necessary for a restaurant procurement and logistics management platform?</t>
+  </si>
+  <si>
+    <t>The system should include several major actors based on the operational flow of the supply chain.
+1. Restaurant Manager
+Responsibilities:
+View ingredient catalog
+Compare suppliers
+Create purchase requests
+Track deliveries
+Confirm goods receipt
+View forecasting dashboards
+2. Supplier Staff
+Responsibilities:
+Publish products
+Manage inventory
+Accept or reject purchase requests
+Prepare shipments
+Generate tracking information
+3. Logistics Dispatcher
+Responsibilities:
+Assign delivery vehicles
+Group delivery orders
+Optimize delivery routes
+Monitor delivery operations
+4. Driver
+Responsibilities:
+Receive delivery tasks
+Navigate delivery routes
+Confirm delivery completion
+5. Platform Administrator
+Responsibilities:
+Manage users
+Approve suppliers
+Monitor KPIs
+Configure optimization rules
+6. AI Optimization Engine
+Responsibilities:
+Forecast demand
+Recommend suppliers
+Predict delays
+Optimize routes
+The use cases should reflect the interaction between these actors and the operational workflow of procurement and logistics management.</t>
+  </si>
+  <si>
+    <t>UI/UX Design</t>
+  </si>
+  <si>
+    <t>How should we organize screen flow and navigation for
+ multiple user roles in a supply chain management platform?</t>
+  </si>
+  <si>
+    <t>The best approach is to use a centralized dashboard architecture where the Home Page acts as the main navigation hub.
+After login:
+users are redirected to role-specific dashboards
+navigation menus are generated based on permissions
+each module contains its own screen hierarchy
+For example:
+Restaurant Manager Flow
+Home Page
+→ Procurement
+→ Forecast Dashboard
+→ Deliveries
+→ Analytics
+Supplier Flow
+Home Page
+→ Products
+→ Inventory
+→ Orders
+→ Shipments
+Logistics Flow
+Home Page
+→ Orders Management
+→ Route Optimization
+→ Vehicle Monitoring
+The screen flow should focus on:
+simple navigation
+minimal screen depth
+clear module separation
+consistent UI structure
+For SRS documentation, the screen flow should represent:
+page-to-page navigation
+screen hierarchy
+movement between modules
+instead of detailed business workflows.</t>
   </si>
 </sst>
 </file>
@@ -585,7 +675,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="409.5">
+    <row r="2" spans="1:4" ht="399">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -639,9 +729,9 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="24.5" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="158" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="41.625" customWidth="1"/>
+    <col min="4" max="4" width="102.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15">
@@ -658,21 +748,33 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" ht="409.5">
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="4"/>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="B2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="409.5">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="4"/>
+      <c r="B3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">

</xml_diff>

<commit_message>
AI Audit log week 3
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenVietKhanh_DE181002.xlsx
+++ b/AI Audit Log_NguyenVietKhanh_DE181002.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\AI_Log\ai-audit-log-KhanhNV1374\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F792AFA-9814-438F-B786-258B6D5AC9A3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F824618-F11A-4F4A-ACD0-F37DDA062F2F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="1" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="11475" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="2" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="34">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -237,6 +237,105 @@
 screen hierarchy
 movement between modules
 instead of detailed business workflows.</t>
+  </si>
+  <si>
+    <t>Database Design</t>
+  </si>
+  <si>
+    <t>What database entities are required for procurement, inventory, logistics, and delivery tracking in a fresh food supply chain system?</t>
+  </si>
+  <si>
+    <t>The database should be organized into several functional domains.
+Authentication &amp; User Management
+Core entities:
+Users
+Roles
+UserSessions
+Notifications
+Restaurant &amp; Supplier Management
+Core entities:
+Restaurants
+Suppliers
+Products
+ProductCategories
+ProductImages
+Procurement Management
+Core entities:
+PurchaseRequests
+PurchaseRequestItems
+SupplierResponses
+These entities support procurement workflows between restaurants and suppliers.
+Inventory Management
+Core entities:
+InventoryStocks
+InventoryMovements
+These tables track realtime inventory quantity and stock history.
+Logistics Management
+Core entities:
+Vehicles
+Drivers
+Routes
+Deliveries
+DeliveryStops
+DeliveryTrackingLogs
+These entities support:
+route management
+delivery assignment
+GPS tracking
+realtime monitoring
+AI &amp; Analytics
+Core entities:
+DemandForecasts
+SupplierRecommendations
+MarketTrends
+RiskAlerts
+These tables store prediction and recommendation data generated by AI modules.
+The relationships between entities should support realtime operational workflows across procurement, inventory, and logistics systems.</t>
+  </si>
+  <si>
+    <t>AI Feature Planning</t>
+  </si>
+  <si>
+    <t>Which AI features are realistic and suitable for a semester-scale fresh food supply chain management project?</t>
+  </si>
+  <si>
+    <t>For a semester-scale project, the AI features should be practical, implementable, and strongly connected to the business domain.
+The most realistic AI features are:
+1. Demand Forecasting
+Predict future ingredient demand using:
+historical procurement data
+seasonal trends
+weather information
+This feature is highly relevant and relatively feasible using models such as Prophet or regression models.
+2. Supplier Recommendation
+Recommend suppliers based on:
+pricing
+delivery performance
+reliability
+rating history
+This can be implemented using scoring algorithms or lightweight recommendation logic.
+3. Route Optimization
+Optimize delivery routes using:
+distance
+traffic conditions
+delivery priority
+Google OR-Tools is suitable for this type of optimization problem.
+4. Delivery Delay Prediction
+Estimate possible delays using:
+traffic data
+weather conditions
+historical delivery duration
+This feature improves delivery planning and operational visibility.
+Complex AI systems such as:
+computer vision
+realtime anomaly detection
+deep learning pipelines
+are generally too difficult for a semester-scale SDLC project unless the team has strong AI specialization and sufficient implementation time.
+The project should prioritize:
+feasibility
+integration quality
+operational usefulness
+instead of overly complex AI experimentation.</t>
   </si>
 </sst>
 </file>
@@ -821,35 +920,61 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" ht="409.5">
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="4"/>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="409.5">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="409.5">
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="409.5">
       <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="4"/>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>33</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>